<commit_message>
cambios a dia 3/09/2025
</commit_message>
<xml_diff>
--- a/archivos_excel/Base_IPMC.xlsx
+++ b/archivos_excel/Base_IPMC.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inegobgt-my.sharepoint.com/personal/diec_ine_gob_gt/Documents/Escritorio/Cambio de base/Power BI/Tablero_SIP_Automatizado/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jdpivaral\WebScraping\solucion\archivos_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{54D89F8C-AC60-4856-BDD7-3550214A9337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A55BA08C-1D89-450C-8749-3F93D25234E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5FE4F3CD-67BA-4DB6-93AE-E83755ABA3ED}"/>
   </bookViews>

</xml_diff>